<commit_message>
added a new file sp152
</commit_message>
<xml_diff>
--- a/June/21.06.2026/northwind.xlsx
+++ b/June/21.06.2026/northwind.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="17760" windowHeight="12380" firstSheet="6" activeTab="13"/>
+    <workbookView windowHeight="17160" firstSheet="6" activeTab="13"/>
   </bookViews>
   <sheets>
     <sheet name="categories" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7231" uniqueCount="1499">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7232" uniqueCount="1500">
   <si>
     <t>categoryid</t>
   </si>
@@ -4540,6 +4540,9 @@
   </si>
   <si>
     <t>Santosh</t>
+  </si>
+  <si>
+    <t>Sum</t>
   </si>
 </sst>
 </file>
@@ -8209,7 +8212,7 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="11.71875" customWidth="1"/>
@@ -8553,6 +8556,23 @@
       <c r="I11">
         <f t="shared" si="1"/>
         <v>51.6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="B12" t="s">
+        <v>1499</v>
+      </c>
+      <c r="C12">
+        <f>SUM(C2:C11)</f>
+        <v>587</v>
+      </c>
+      <c r="H12">
+        <f>SUM(H2:H11)</f>
+        <v>3282</v>
+      </c>
+      <c r="I12">
+        <f>SUM(I2:I11)</f>
+        <v>656.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>